<commit_message>
Add PMIC chapter with commercial converter block diagrams, rename NVC sweep plots
New chapter covers PMIC options (AEM10941/13920, SPV1040/1050, bq25570)
with their block diagrams; NVC_sweep plot files renamed from Y_* to NVC_*
for consistency, plus new OCV data files.
</commit_message>
<xml_diff>
--- a/Matlab/Data Processing/NVC/NVC_OCV.xlsx
+++ b/Matlab/Data Processing/NVC/NVC_OCV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNIPD\Magistrale\Master Thesis\Matlab\Data Processing\NVC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A3C71AA-8A64-4B95-9315-D086639F03C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0908E155-A9E1-4142-A042-00E1F9B8E92E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,12 +25,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
   <si>
     <t>R = inf</t>
-  </si>
-  <si>
-    <t>CL = 430 uF</t>
   </si>
   <si>
     <t>V</t>
@@ -401,32 +398,29 @@
   <sheetData>
     <row r="4" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
         <v>0</v>
       </c>
-      <c r="D4" t="s">
-        <v>1</v>
-      </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.3">
       <c r="D5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" t="s">
         <v>3</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>4</v>
-      </c>
-      <c r="E6" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.3">
@@ -434,10 +428,10 @@
         <v>100</v>
       </c>
       <c r="D7" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" t="s">
         <v>6</v>
-      </c>
-      <c r="E7" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.3">
@@ -445,10 +439,10 @@
         <v>150</v>
       </c>
       <c r="D8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
         <v>8</v>
-      </c>
-      <c r="E8" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.3">
@@ -456,10 +450,10 @@
         <v>200</v>
       </c>
       <c r="D9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" t="s">
         <v>10</v>
-      </c>
-      <c r="E9" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.3">
@@ -467,10 +461,10 @@
         <v>250</v>
       </c>
       <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
         <v>12</v>
-      </c>
-      <c r="E10" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.3">
@@ -478,10 +472,10 @@
         <v>300</v>
       </c>
       <c r="D11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
@@ -489,10 +483,10 @@
         <v>350</v>
       </c>
       <c r="D12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.3">
@@ -500,10 +494,10 @@
         <v>400</v>
       </c>
       <c r="D13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>